<commit_message>
Add Excercise 3A and 1A getting set up
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aspennerhoden\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B4F32A-4F22-4D62-B31F-94E13D087977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3403A54-42B8-4997-B303-80DFD9FEB745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8D22D330-DD29-49E6-AE16-8B90DAC48831}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Name of data source</t>
   </si>
@@ -579,6 +579,9 @@
       <c r="E4" t="s">
         <v>24</v>
       </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
       <c r="G4" t="s">
         <v>19</v>
       </c>

</xml_diff>